<commit_message>
bilder vom projekt hinzugefügt überall
</commit_message>
<xml_diff>
--- a/LaTeXTemplate/Bewertungsschema.xlsx
+++ b/LaTeXTemplate/Bewertungsschema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlm\Documents\LaTeXTemplate\LaTeXTemplate\LaTeXTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFECEAB-3531-405B-8776-4630E92E6108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44581FCF-300B-4CDB-A511-8F47AEB08FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -277,12 +277,6 @@
     <t>Delighters</t>
   </si>
   <si>
-    <t>Delighter 5</t>
-  </si>
-  <si>
-    <t>Delighter 6</t>
-  </si>
-  <si>
     <t>Delighter 7</t>
   </si>
   <si>
@@ -1031,6 +1025,12 @@
   </si>
   <si>
     <t>NB-Stud</t>
+  </si>
+  <si>
+    <t>7 eigene tikz-Zeichnungen in der Demontageanleitung</t>
+  </si>
+  <si>
+    <t>10 eigene tikz Zeichnungen in Montageanleitung</t>
   </si>
 </sst>
 </file>
@@ -1243,7 +1243,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1273,6 +1273,22 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1290,25 +1306,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1615,31 +1612,31 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="63.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="23" t="s">
-        <v>271</v>
-      </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
+      <c r="A7" s="29" t="s">
+        <v>269</v>
+      </c>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
     </row>
     <row r="9" spans="1:8" ht="28.5" x14ac:dyDescent="0.85">
       <c r="A9" s="2" t="s">
@@ -1647,131 +1644,131 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E10" s="31" t="s">
-        <v>270</v>
-      </c>
-      <c r="F10" s="32"/>
+      <c r="E10" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="F10" s="26"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="26" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" s="26">
+        <v>7024847</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="E11" s="28" t="s">
+        <v>286</v>
+      </c>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A12" s="26" t="s">
         <v>273</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B12" s="26" t="s">
         <v>274</v>
       </c>
-      <c r="C11" s="34">
-        <v>7024847</v>
-      </c>
-      <c r="D11" s="34" t="s">
-        <v>298</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>288</v>
-      </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A12" s="32" t="s">
+      <c r="C12" s="26">
+        <v>7024769</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>285</v>
+      </c>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A13" s="26" t="s">
         <v>275</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B13" s="26" t="s">
         <v>276</v>
       </c>
-      <c r="C12" s="32">
-        <v>7024769</v>
-      </c>
-      <c r="D12" s="32" t="s">
-        <v>291</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>287</v>
-      </c>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A13" s="34" t="s">
+      <c r="C13" s="26">
+        <v>7024749</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="E13" s="28" t="s">
+        <v>284</v>
+      </c>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A14" s="26" t="s">
         <v>277</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B14" s="26" t="s">
         <v>278</v>
       </c>
-      <c r="C13" s="34">
-        <v>7024749</v>
-      </c>
-      <c r="D13" s="32" t="s">
-        <v>296</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>286</v>
-      </c>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A14" s="34" t="s">
+      <c r="C14" s="26">
+        <v>7025068</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>295</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>283</v>
+      </c>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A15" s="26" t="s">
         <v>279</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B15" s="26" t="s">
         <v>280</v>
       </c>
-      <c r="C14" s="32">
-        <v>7025068</v>
-      </c>
-      <c r="D14" s="32" t="s">
-        <v>297</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>285</v>
-      </c>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A15" s="34" t="s">
+      <c r="C15" s="26">
+        <v>7024640</v>
+      </c>
+      <c r="D15" s="26" t="s">
         <v>281</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="E15" s="28" t="s">
         <v>282</v>
       </c>
-      <c r="C15" s="32">
-        <v>7024640</v>
-      </c>
-      <c r="D15" s="32" t="s">
-        <v>283</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>284</v>
-      </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="32"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B17" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="24" t="s">
         <v>44</v>
       </c>
       <c r="E17" s="3"/>
@@ -1780,13 +1777,13 @@
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="24" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B21" s="4">
         <v>45727</v>
@@ -1794,17 +1791,17 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="29">
+        <v>76</v>
+      </c>
+      <c r="B22" s="23">
         <v>45831</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24" s="24" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1818,20 +1815,20 @@
     </row>
     <row r="28" spans="1:6" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A28" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -1843,7 +1840,7 @@
     <row r="33" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A33" s="7"/>
       <c r="B33" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -1855,7 +1852,7 @@
     <row r="34" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A34" s="8"/>
       <c r="B34" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -1867,7 +1864,7 @@
     <row r="35" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A35" s="8"/>
       <c r="B35" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -1879,7 +1876,7 @@
     <row r="36" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A36" s="8"/>
       <c r="B36" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -1903,10 +1900,10 @@
     <row r="38" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A38" s="7"/>
       <c r="B38" s="8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D38" s="8"/>
       <c r="E38" s="8">
@@ -1920,7 +1917,7 @@
       <c r="A39" s="7"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
@@ -1932,7 +1929,7 @@
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8"/>
@@ -1944,7 +1941,7 @@
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8">
@@ -1958,7 +1955,7 @@
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8">
@@ -1972,7 +1969,7 @@
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8"/>
@@ -1984,7 +1981,7 @@
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
@@ -1997,7 +1994,7 @@
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
       <c r="D45" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E45" s="15">
         <f>-SUM(E32:E44)</f>
@@ -2017,44 +2014,44 @@
     </row>
     <row r="48" spans="1:12" s="5" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K48"/>
       <c r="L48"/>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8"/>
       <c r="F49" s="8">
         <v>10</v>
       </c>
-      <c r="G49" s="24" t="s">
+      <c r="G49" s="30" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A50" s="7"/>
       <c r="B50" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
       <c r="F50" s="8">
         <v>5</v>
       </c>
-      <c r="G50" s="24"/>
+      <c r="G50" s="30"/>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A51" s="7"/>
@@ -2067,72 +2064,72 @@
       <c r="F51" s="8">
         <v>5</v>
       </c>
-      <c r="G51" s="24"/>
+      <c r="G51" s="30"/>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A52" s="7"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8"/>
       <c r="F52" s="8">
         <v>5</v>
       </c>
-      <c r="G52" s="24"/>
+      <c r="G52" s="30"/>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A53" s="7"/>
       <c r="B53" s="7"/>
       <c r="C53" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8"/>
       <c r="F53" s="8">
         <v>10</v>
       </c>
-      <c r="G53" s="24"/>
+      <c r="G53" s="30"/>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A54" s="8"/>
       <c r="B54" s="7"/>
       <c r="C54" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
       <c r="F54" s="8">
         <v>25</v>
       </c>
-      <c r="G54" s="24"/>
+      <c r="G54" s="30"/>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A55" s="7"/>
       <c r="B55" s="7"/>
       <c r="C55" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
       <c r="F55" s="8">
         <v>5</v>
       </c>
-      <c r="G55" s="24"/>
+      <c r="G55" s="30"/>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A56" s="7"/>
       <c r="B56" s="7"/>
       <c r="C56" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
       <c r="F56" s="8">
         <v>5</v>
       </c>
-      <c r="G56" s="24"/>
+      <c r="G56" s="30"/>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A57" s="7"/>
@@ -2145,75 +2142,75 @@
       <c r="F57" s="8">
         <v>10</v>
       </c>
-      <c r="G57" s="24"/>
+      <c r="G57" s="30"/>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A58" s="7"/>
       <c r="B58" s="7"/>
       <c r="C58" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D58" s="8"/>
       <c r="E58" s="8"/>
       <c r="F58" s="8">
         <v>5</v>
       </c>
-      <c r="G58" s="24"/>
+      <c r="G58" s="30"/>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A59" s="7"/>
       <c r="B59" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D59" s="8"/>
       <c r="E59" s="8"/>
       <c r="F59" s="8">
         <v>5</v>
       </c>
-      <c r="G59" s="24"/>
+      <c r="G59" s="30"/>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A60" s="7"/>
       <c r="B60" s="7"/>
       <c r="C60" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D60" s="8"/>
       <c r="E60" s="8"/>
       <c r="F60" s="8">
         <v>20</v>
       </c>
-      <c r="G60" s="24"/>
+      <c r="G60" s="30"/>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A61" s="7"/>
       <c r="B61" s="7"/>
       <c r="C61" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D61" s="8"/>
       <c r="E61" s="8"/>
       <c r="F61" s="8">
         <v>10</v>
       </c>
-      <c r="G61" s="24"/>
+      <c r="G61" s="30"/>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A62" s="7"/>
       <c r="B62" s="7"/>
       <c r="C62" s="8"/>
       <c r="D62" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E62" s="15">
         <f>-SUM(E49:E61)</f>
         <v>0</v>
       </c>
       <c r="F62" s="8"/>
-      <c r="G62" s="24"/>
+      <c r="G62" s="30"/>
     </row>
     <row r="63" spans="1:13" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="1"/>
@@ -2231,7 +2228,7 @@
     </row>
     <row r="64" spans="1:13" s="5" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K64"/>
       <c r="L64"/>
@@ -2242,10 +2239,10 @@
         <v>Montageanleitung</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D65" s="8"/>
       <c r="E65" s="8"/>
@@ -2256,10 +2253,10 @@
     <row r="66" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A66" s="7"/>
       <c r="B66" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D66" s="8"/>
       <c r="E66" s="8"/>
@@ -2271,7 +2268,7 @@
       <c r="A67" s="7"/>
       <c r="B67" s="7"/>
       <c r="C67" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D67" s="8"/>
       <c r="E67" s="8"/>
@@ -2283,7 +2280,7 @@
       <c r="A68" s="7"/>
       <c r="B68" s="7"/>
       <c r="C68" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D68" s="8"/>
       <c r="E68" s="8"/>
@@ -2295,7 +2292,7 @@
       <c r="A69" s="7"/>
       <c r="B69" s="7"/>
       <c r="C69" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D69" s="8"/>
       <c r="E69" s="8"/>
@@ -2307,7 +2304,7 @@
       <c r="A70" s="7"/>
       <c r="B70" s="7"/>
       <c r="C70" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D70" s="8"/>
       <c r="E70" s="8"/>
@@ -2319,7 +2316,7 @@
       <c r="A71" s="7"/>
       <c r="B71" s="7"/>
       <c r="C71" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D71" s="8"/>
       <c r="E71" s="8"/>
@@ -2332,7 +2329,7 @@
       <c r="B72" s="7"/>
       <c r="C72" s="8"/>
       <c r="D72" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E72" s="15">
         <f>-SUM(E65:E71)</f>
@@ -2357,20 +2354,20 @@
     </row>
     <row r="75" spans="1:12" s="5" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K75"/>
       <c r="L75"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A76" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C76" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="B76" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C76" s="8" t="s">
-        <v>105</v>
       </c>
       <c r="D76" s="8"/>
       <c r="E76" s="8"/>
@@ -2381,10 +2378,10 @@
     <row r="77" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A77" s="7"/>
       <c r="B77" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D77" s="8"/>
       <c r="E77" s="8"/>
@@ -2396,7 +2393,7 @@
       <c r="A78" s="7"/>
       <c r="B78" s="7"/>
       <c r="C78" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D78" s="8"/>
       <c r="E78" s="8"/>
@@ -2408,7 +2405,7 @@
       <c r="A79" s="7"/>
       <c r="B79" s="7"/>
       <c r="C79" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D79" s="8"/>
       <c r="E79" s="8"/>
@@ -2420,7 +2417,7 @@
       <c r="A80" s="7"/>
       <c r="B80" s="7"/>
       <c r="C80" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D80" s="8"/>
       <c r="E80" s="8"/>
@@ -2432,7 +2429,7 @@
       <c r="A81" s="7"/>
       <c r="B81" s="7"/>
       <c r="C81" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D81" s="8"/>
       <c r="E81" s="8"/>
@@ -2444,7 +2441,7 @@
       <c r="A82" s="7"/>
       <c r="B82" s="7"/>
       <c r="C82" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D82" s="8"/>
       <c r="E82" s="8"/>
@@ -2457,7 +2454,7 @@
       <c r="B83" s="7"/>
       <c r="C83" s="8"/>
       <c r="D83" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E83" s="15">
         <f>-SUM(E76:E82)</f>
@@ -2490,10 +2487,10 @@
         <v>34</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D87" s="8"/>
       <c r="E87" s="8"/>
@@ -2505,7 +2502,7 @@
       <c r="A88" s="7"/>
       <c r="B88" s="8"/>
       <c r="C88" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D88" s="8"/>
       <c r="E88" s="8"/>
@@ -2517,7 +2514,7 @@
       <c r="A89" s="7"/>
       <c r="B89" s="8"/>
       <c r="C89" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D89" s="8"/>
       <c r="E89" s="8"/>
@@ -2528,10 +2525,10 @@
     <row r="90" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A90" s="7"/>
       <c r="B90" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D90" s="8"/>
       <c r="E90" s="8"/>
@@ -2543,7 +2540,7 @@
       <c r="A91" s="7"/>
       <c r="B91" s="7"/>
       <c r="C91" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D91" s="8"/>
       <c r="E91" s="8"/>
@@ -2555,7 +2552,7 @@
       <c r="A92" s="7"/>
       <c r="B92" s="7"/>
       <c r="C92" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D92" s="8"/>
       <c r="E92" s="8"/>
@@ -2567,7 +2564,7 @@
       <c r="A93" s="7"/>
       <c r="B93" s="7"/>
       <c r="C93" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D93" s="8"/>
       <c r="E93" s="8"/>
@@ -2580,7 +2577,7 @@
       <c r="B94" s="7"/>
       <c r="C94" s="7"/>
       <c r="D94" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E94" s="15">
         <f>-SUM(E87:E93)</f>
@@ -2605,18 +2602,18 @@
     </row>
     <row r="97" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A98" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D98" s="8"/>
       <c r="E98" s="8"/>
@@ -2628,7 +2625,7 @@
       <c r="A99" s="7"/>
       <c r="B99" s="8"/>
       <c r="C99" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D99" s="8"/>
       <c r="E99" s="8"/>
@@ -2639,10 +2636,10 @@
     <row r="100" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A100" s="7"/>
       <c r="B100" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D100" s="8"/>
       <c r="E100" s="8"/>
@@ -2654,7 +2651,7 @@
       <c r="A101" s="7"/>
       <c r="B101" s="7"/>
       <c r="C101" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D101" s="8"/>
       <c r="E101" s="8"/>
@@ -2667,7 +2664,7 @@
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
       <c r="D102" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E102" s="15">
         <f>-SUM(E98:E101)</f>
@@ -2693,18 +2690,18 @@
     </row>
     <row r="105" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A106" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D106" s="8"/>
       <c r="E106" s="8">
@@ -2717,10 +2714,10 @@
     <row r="107" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A107" s="7"/>
       <c r="B107" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D107" s="8"/>
       <c r="E107" s="8"/>
@@ -2732,7 +2729,7 @@
       <c r="A108" s="7"/>
       <c r="B108" s="7"/>
       <c r="C108" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D108" s="8"/>
       <c r="E108" s="8"/>
@@ -2744,7 +2741,7 @@
       <c r="A109" s="7"/>
       <c r="B109" s="7"/>
       <c r="C109" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D109" s="8"/>
       <c r="E109" s="8"/>
@@ -2757,7 +2754,7 @@
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
       <c r="D110" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E110" s="15">
         <f>-SUM(E107:E109)</f>
@@ -2783,18 +2780,18 @@
     </row>
     <row r="113" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A114" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D114" s="8"/>
       <c r="E114" s="8">
@@ -2807,10 +2804,10 @@
     <row r="115" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A115" s="7"/>
       <c r="B115" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D115" s="8"/>
       <c r="E115" s="8"/>
@@ -2822,7 +2819,7 @@
       <c r="A116" s="7"/>
       <c r="B116" s="7"/>
       <c r="C116" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D116" s="8"/>
       <c r="E116" s="8"/>
@@ -2834,7 +2831,7 @@
       <c r="A117" s="7"/>
       <c r="B117" s="7"/>
       <c r="C117" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D117" s="8"/>
       <c r="E117" s="8"/>
@@ -2847,7 +2844,7 @@
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
       <c r="D118" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E118" s="15">
         <f>-SUM(E115:E117)</f>
@@ -2870,21 +2867,21 @@
     <row r="120" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="121" spans="1:6" ht="21" x14ac:dyDescent="0.65">
       <c r="A121" s="16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A123" s="7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B123" s="7"/>
       <c r="C123" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D123" s="8"/>
       <c r="E123" s="8"/>
@@ -2896,7 +2893,7 @@
       <c r="A124" s="8"/>
       <c r="B124" s="8"/>
       <c r="C124" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D124" s="8"/>
       <c r="E124" s="8">
@@ -2910,7 +2907,7 @@
       <c r="A125" s="8"/>
       <c r="B125" s="8"/>
       <c r="C125" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D125" s="8"/>
       <c r="E125" s="8"/>
@@ -2922,7 +2919,7 @@
       <c r="A126" s="8"/>
       <c r="B126" s="8"/>
       <c r="C126" s="8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D126" s="8"/>
       <c r="E126" s="8"/>
@@ -2934,7 +2931,7 @@
       <c r="A127" s="8"/>
       <c r="B127" s="8"/>
       <c r="C127" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D127" s="8"/>
       <c r="E127" s="8"/>
@@ -2946,7 +2943,7 @@
       <c r="A128" s="8"/>
       <c r="B128" s="8"/>
       <c r="C128" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D128" s="8"/>
       <c r="E128" s="8"/>
@@ -2959,7 +2956,7 @@
       <c r="B129" s="8"/>
       <c r="C129" s="8"/>
       <c r="D129" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E129" s="15">
         <f>-SUM(E123:E128)</f>
@@ -2979,15 +2976,15 @@
     </row>
     <row r="131" spans="1:7" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A131" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A132" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B132" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="B132" s="8" t="s">
-        <v>119</v>
       </c>
       <c r="C132" s="8"/>
       <c r="D132" s="8"/>
@@ -2999,7 +2996,7 @@
     <row r="133" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A133" s="7"/>
       <c r="B133" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C133" s="8"/>
       <c r="D133" s="8"/>
@@ -3011,7 +3008,7 @@
     <row r="134" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A134" s="8"/>
       <c r="B134" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C134" s="8"/>
       <c r="D134" s="8"/>
@@ -3025,7 +3022,7 @@
       <c r="B135" s="19"/>
       <c r="C135" s="8"/>
       <c r="D135" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E135" s="15">
         <f>-SUM(E132:E134)</f>
@@ -3045,13 +3042,13 @@
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A139" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D139" s="8"/>
       <c r="E139" s="8" t="s">
@@ -3065,7 +3062,7 @@
       <c r="A140" s="8"/>
       <c r="B140" s="8"/>
       <c r="C140" s="8" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D140" s="8"/>
       <c r="E140" s="8" t="s">
@@ -3074,17 +3071,17 @@
       <c r="F140" s="8">
         <v>10</v>
       </c>
-      <c r="G140" s="25" t="s">
+      <c r="G140" s="31" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A141" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B141" s="8"/>
       <c r="C141" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D141" s="8"/>
       <c r="E141" s="8" t="s">
@@ -3093,13 +3090,13 @@
       <c r="F141" s="8">
         <v>10</v>
       </c>
-      <c r="G141" s="25"/>
+      <c r="G141" s="31"/>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A142" s="8"/>
       <c r="B142" s="8"/>
       <c r="C142" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D142" s="8"/>
       <c r="E142" s="8" t="s">
@@ -3108,13 +3105,13 @@
       <c r="F142" s="8">
         <v>10</v>
       </c>
-      <c r="G142" s="25"/>
+      <c r="G142" s="31"/>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A143" s="8"/>
       <c r="B143" s="8"/>
       <c r="C143" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D143" s="8"/>
       <c r="E143" s="8" t="s">
@@ -3123,13 +3120,13 @@
       <c r="F143" s="8">
         <v>10</v>
       </c>
-      <c r="G143" s="25"/>
+      <c r="G143" s="31"/>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A144" s="7"/>
       <c r="B144" s="8"/>
       <c r="C144" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="8" t="s">
@@ -3138,16 +3135,16 @@
       <c r="F144" s="8">
         <v>50</v>
       </c>
-      <c r="G144" s="25"/>
+      <c r="G144" s="31"/>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A145" s="8"/>
       <c r="B145" s="8"/>
       <c r="C145" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D145" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E145" s="8" t="s">
         <v>35</v>
@@ -3155,13 +3152,13 @@
       <c r="F145" s="8">
         <v>30</v>
       </c>
-      <c r="G145" s="25"/>
+      <c r="G145" s="31"/>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A146" s="7"/>
       <c r="B146" s="8"/>
       <c r="C146" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D146" s="8"/>
       <c r="E146" s="8" t="s">
@@ -3170,21 +3167,21 @@
       <c r="F146" s="8">
         <v>40</v>
       </c>
-      <c r="G146" s="25"/>
+      <c r="G146" s="31"/>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A147" s="8"/>
       <c r="B147" s="8"/>
       <c r="C147" s="8"/>
       <c r="D147" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E147" s="15">
         <f>-SUM(E140:E146)</f>
         <v>0</v>
       </c>
       <c r="F147" s="8"/>
-      <c r="G147" s="25"/>
+      <c r="G147" s="31"/>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.45">
       <c r="E148">
@@ -3194,18 +3191,18 @@
       <c r="F148">
         <v>170</v>
       </c>
-      <c r="G148" s="25"/>
+      <c r="G148" s="31"/>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="G149" s="25"/>
+      <c r="G149" s="31"/>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A150" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B150" s="8"/>
       <c r="C150" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D150" s="8"/>
       <c r="E150" s="8" t="s">
@@ -3214,41 +3211,41 @@
       <c r="F150" s="8">
         <v>10</v>
       </c>
-      <c r="G150" s="25"/>
+      <c r="G150" s="31"/>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A151" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B151" s="8"/>
       <c r="C151" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D151" s="8"/>
       <c r="E151" s="8"/>
       <c r="F151" s="8">
         <v>10</v>
       </c>
-      <c r="G151" s="25"/>
+      <c r="G151" s="31"/>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A152" s="7"/>
       <c r="B152" s="8"/>
       <c r="C152" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D152" s="8"/>
       <c r="E152" s="8"/>
       <c r="F152" s="8">
         <v>10</v>
       </c>
-      <c r="G152" s="25"/>
+      <c r="G152" s="31"/>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A153" s="7"/>
       <c r="B153" s="8"/>
       <c r="C153" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D153" s="8"/>
       <c r="E153" s="8" t="s">
@@ -3257,13 +3254,13 @@
       <c r="F153" s="8">
         <v>10</v>
       </c>
-      <c r="G153" s="25"/>
+      <c r="G153" s="31"/>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A154" s="8"/>
       <c r="B154" s="8"/>
       <c r="C154" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D154" s="8"/>
       <c r="E154" s="8" t="s">
@@ -3272,13 +3269,13 @@
       <c r="F154" s="8">
         <v>15</v>
       </c>
-      <c r="G154" s="25"/>
+      <c r="G154" s="31"/>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A155" s="8"/>
       <c r="B155" s="8"/>
       <c r="C155" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D155" s="8"/>
       <c r="E155" s="8" t="s">
@@ -3287,13 +3284,13 @@
       <c r="F155" s="8">
         <v>10</v>
       </c>
-      <c r="G155" s="25"/>
+      <c r="G155" s="31"/>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A156" s="8"/>
       <c r="B156" s="8"/>
       <c r="C156" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D156" s="8"/>
       <c r="E156" s="8" t="s">
@@ -3302,7 +3299,7 @@
       <c r="F156" s="8">
         <v>15</v>
       </c>
-      <c r="G156" s="25"/>
+      <c r="G156" s="31"/>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A157" s="8"/>
@@ -3315,26 +3312,26 @@
       <c r="F157" s="8">
         <v>15</v>
       </c>
-      <c r="G157" s="25"/>
+      <c r="G157" s="31"/>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A158" s="8"/>
       <c r="B158" s="8"/>
       <c r="C158" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D158" s="8"/>
       <c r="E158" s="8"/>
       <c r="F158" s="8">
         <v>5</v>
       </c>
-      <c r="G158" s="25"/>
+      <c r="G158" s="31"/>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A159" s="8"/>
       <c r="B159" s="8"/>
       <c r="C159" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D159" s="8"/>
       <c r="E159" s="8">
@@ -3343,21 +3340,21 @@
       <c r="F159" s="8">
         <v>0</v>
       </c>
-      <c r="G159" s="25"/>
+      <c r="G159" s="31"/>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A160" s="8"/>
       <c r="B160" s="8"/>
       <c r="C160" s="8"/>
       <c r="D160" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E160" s="15">
         <f>-SUM(E150:E158)</f>
         <v>0</v>
       </c>
       <c r="F160" s="8"/>
-      <c r="G160" s="25"/>
+      <c r="G160" s="31"/>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.45">
       <c r="E161">
@@ -3368,10 +3365,10 @@
         <f>SUM(F150:F159)</f>
         <v>100</v>
       </c>
-      <c r="G161" s="25"/>
+      <c r="G161" s="31"/>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="G162" s="25"/>
+      <c r="G162" s="31"/>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A163" s="7" t="str">
@@ -3391,7 +3388,7 @@
         <f t="shared" ref="F163:F171" si="1">F150</f>
         <v>10</v>
       </c>
-      <c r="G163" s="25"/>
+      <c r="G163" s="31"/>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A164" s="8" t="str">
@@ -3411,7 +3408,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="G164" s="25"/>
+      <c r="G164" s="31"/>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A165" s="8"/>
@@ -3428,7 +3425,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="G165" s="25"/>
+      <c r="G165" s="31"/>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A166" s="7"/>
@@ -3445,7 +3442,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="G166" s="25"/>
+      <c r="G166" s="31"/>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A167" s="7"/>
@@ -3462,7 +3459,7 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="G167" s="25"/>
+      <c r="G167" s="31"/>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A168" s="7"/>
@@ -3477,7 +3474,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="G168" s="25"/>
+      <c r="G168" s="31"/>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A169" s="7"/>
@@ -3494,7 +3491,7 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="G169" s="25"/>
+      <c r="G169" s="31"/>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A170" s="8"/>
@@ -3511,7 +3508,7 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="G170" s="25"/>
+      <c r="G170" s="31"/>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A171" s="8"/>
@@ -3526,7 +3523,7 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="G171" s="25"/>
+      <c r="G171" s="31"/>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A172" s="8"/>
@@ -3544,21 +3541,21 @@
         <f t="shared" ref="F172" si="3">F159</f>
         <v>0</v>
       </c>
-      <c r="G172" s="25"/>
+      <c r="G172" s="31"/>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A173" s="8"/>
       <c r="B173" s="8"/>
       <c r="C173" s="8"/>
       <c r="D173" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E173" s="15">
         <f>-SUM(E163:E171)</f>
         <v>0</v>
       </c>
       <c r="F173" s="8"/>
-      <c r="G173" s="25"/>
+      <c r="G173" s="31"/>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.45">
       <c r="E174">
@@ -3569,7 +3566,7 @@
         <f>SUM(F163:F172)</f>
         <v>100</v>
       </c>
-      <c r="G174" s="25"/>
+      <c r="G174" s="31"/>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A175" s="7" t="str">
@@ -3587,7 +3584,7 @@
         <f t="shared" ref="F175:F183" si="5">F163</f>
         <v>10</v>
       </c>
-      <c r="G175" s="25"/>
+      <c r="G175" s="31"/>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A176" s="7" t="str">
@@ -3605,7 +3602,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="G176" s="25"/>
+      <c r="G176" s="31"/>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A177" s="7"/>
@@ -3620,7 +3617,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="G177" s="25"/>
+      <c r="G177" s="31"/>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A178" s="7"/>
@@ -3635,7 +3632,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="G178" s="25"/>
+      <c r="G178" s="31"/>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A179" s="7"/>
@@ -3650,7 +3647,7 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="G179" s="25"/>
+      <c r="G179" s="31"/>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A180" s="7"/>
@@ -3665,7 +3662,7 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="G180" s="25"/>
+      <c r="G180" s="31"/>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A181" s="7"/>
@@ -3680,7 +3677,7 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="G181" s="25"/>
+      <c r="G181" s="31"/>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A182" s="7"/>
@@ -3695,7 +3692,7 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="G182" s="25"/>
+      <c r="G182" s="31"/>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A183" s="7"/>
@@ -3710,7 +3707,7 @@
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="G183" s="25"/>
+      <c r="G183" s="31"/>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A184" s="7"/>
@@ -3728,21 +3725,21 @@
         <f t="shared" ref="F184" si="7">F172</f>
         <v>0</v>
       </c>
-      <c r="G184" s="25"/>
+      <c r="G184" s="31"/>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A185" s="7"/>
       <c r="B185" s="7"/>
       <c r="C185" s="8"/>
       <c r="D185" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E185" s="15">
         <f>-SUM(E175:E183)</f>
         <v>0</v>
       </c>
       <c r="F185" s="8"/>
-      <c r="G185" s="25"/>
+      <c r="G185" s="31"/>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A186" s="1"/>
@@ -3755,15 +3752,15 @@
         <f>SUM(F175:F184)</f>
         <v>100</v>
       </c>
-      <c r="G186" s="25"/>
+      <c r="G186" s="31"/>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A187" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B187" s="8"/>
       <c r="C187" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D187" s="8"/>
       <c r="E187" s="8" t="s">
@@ -3772,59 +3769,59 @@
       <c r="F187" s="8">
         <v>10</v>
       </c>
-      <c r="G187" s="25"/>
+      <c r="G187" s="31"/>
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A188" s="7"/>
       <c r="B188" s="8"/>
       <c r="C188" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D188" s="8"/>
       <c r="E188" s="8"/>
       <c r="F188" s="8">
         <v>10</v>
       </c>
-      <c r="G188" s="25"/>
+      <c r="G188" s="31"/>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A189" s="7"/>
       <c r="B189" s="8"/>
       <c r="C189" s="8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D189" s="8"/>
       <c r="E189" s="8"/>
       <c r="F189" s="8">
         <v>10</v>
       </c>
-      <c r="G189" s="25"/>
+      <c r="G189" s="31"/>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A190" s="7"/>
       <c r="B190" s="8"/>
       <c r="C190" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D190" s="8"/>
       <c r="E190" s="8"/>
       <c r="F190" s="8">
         <v>10</v>
       </c>
-      <c r="G190" s="25"/>
+      <c r="G190" s="31"/>
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A191" s="7"/>
       <c r="B191" s="8"/>
       <c r="C191" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D191" s="8"/>
       <c r="E191" s="8"/>
       <c r="F191" s="8">
         <v>10</v>
       </c>
-      <c r="G191" s="25"/>
+      <c r="G191" s="31"/>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A192" s="7"/>
@@ -3837,29 +3834,29 @@
       <c r="F192" s="8">
         <v>10</v>
       </c>
-      <c r="G192" s="25"/>
+      <c r="G192" s="31"/>
     </row>
     <row r="193" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A193" s="7"/>
       <c r="B193" s="8"/>
       <c r="C193" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D193" s="8"/>
       <c r="E193" s="8"/>
       <c r="F193" s="8">
         <v>10</v>
       </c>
-      <c r="G193" s="25"/>
+      <c r="G193" s="31"/>
     </row>
     <row r="194" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A194" s="7"/>
       <c r="B194" s="8"/>
       <c r="C194" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E194" s="8" t="s">
         <v>35</v>
@@ -3867,13 +3864,13 @@
       <c r="F194" s="8">
         <v>10</v>
       </c>
-      <c r="G194" s="25"/>
+      <c r="G194" s="31"/>
     </row>
     <row r="195" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A195" s="8"/>
       <c r="B195" s="8"/>
       <c r="C195" s="8" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D195" s="8"/>
       <c r="E195" s="8" t="s">
@@ -3882,13 +3879,13 @@
       <c r="F195" s="8">
         <v>10</v>
       </c>
-      <c r="G195" s="25"/>
+      <c r="G195" s="31"/>
     </row>
     <row r="196" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A196" s="8"/>
       <c r="B196" s="8"/>
       <c r="C196" s="8" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D196" s="8"/>
       <c r="E196" s="8" t="s">
@@ -3897,13 +3894,13 @@
       <c r="F196" s="8">
         <v>5</v>
       </c>
-      <c r="G196" s="25"/>
+      <c r="G196" s="31"/>
     </row>
     <row r="197" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A197" s="8"/>
       <c r="B197" s="8"/>
       <c r="C197" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D197" s="8"/>
       <c r="E197" s="8" t="s">
@@ -3912,21 +3909,21 @@
       <c r="F197" s="8">
         <v>5</v>
       </c>
-      <c r="G197" s="25"/>
+      <c r="G197" s="31"/>
     </row>
     <row r="198" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A198" s="8"/>
       <c r="B198" s="8"/>
       <c r="C198" s="8"/>
       <c r="D198" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E198" s="15">
         <f>-SUM(E187:E197)</f>
         <v>0</v>
       </c>
       <c r="F198" s="8"/>
-      <c r="G198" s="25"/>
+      <c r="G198" s="31"/>
     </row>
     <row r="199" spans="1:12" x14ac:dyDescent="0.45">
       <c r="E199">
@@ -3937,14 +3934,14 @@
         <f>SUM(F187:F197)</f>
         <v>100</v>
       </c>
-      <c r="G199" s="25"/>
+      <c r="G199" s="31"/>
     </row>
     <row r="200" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="G200" s="25"/>
+      <c r="G200" s="31"/>
     </row>
     <row r="201" spans="1:12" s="5" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A201" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K201"/>
       <c r="L201"/>
@@ -3954,11 +3951,11 @@
     </row>
     <row r="203" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A203" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B203" s="7"/>
       <c r="C203" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D203" s="8"/>
       <c r="E203" s="8"/>
@@ -3970,7 +3967,7 @@
       <c r="A204" s="8"/>
       <c r="B204" s="8"/>
       <c r="C204" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D204" s="8"/>
       <c r="E204" s="8"/>
@@ -3982,7 +3979,7 @@
       <c r="A205" s="8"/>
       <c r="B205" s="8"/>
       <c r="C205" s="8" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D205" s="8"/>
       <c r="E205" s="8"/>
@@ -3994,7 +3991,7 @@
       <c r="A206" s="8"/>
       <c r="B206" s="8"/>
       <c r="C206" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D206" s="8"/>
       <c r="E206" s="8"/>
@@ -4006,7 +4003,7 @@
       <c r="A207" s="8"/>
       <c r="B207" s="8"/>
       <c r="C207" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D207" s="8"/>
       <c r="E207" s="8"/>
@@ -4018,7 +4015,7 @@
       <c r="A208" s="8"/>
       <c r="B208" s="8"/>
       <c r="C208" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D208" s="8"/>
       <c r="E208" s="8"/>
@@ -4030,7 +4027,7 @@
       <c r="A209" s="8"/>
       <c r="B209" s="8"/>
       <c r="C209" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D209" s="8"/>
       <c r="E209" s="8"/>
@@ -4043,7 +4040,7 @@
       <c r="B210" s="8"/>
       <c r="C210" s="8"/>
       <c r="D210" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E210" s="15">
         <f>-SUM(E203:E209)</f>
@@ -4063,12 +4060,12 @@
     </row>
     <row r="213" spans="1:7" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A213" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A214" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B214" s="7"/>
       <c r="C214" s="8" t="s">
@@ -4079,7 +4076,7 @@
       <c r="F214" s="8">
         <v>5</v>
       </c>
-      <c r="G214" s="26" t="s">
+      <c r="G214" s="32" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4089,14 +4086,14 @@
       </c>
       <c r="B215" s="7"/>
       <c r="C215" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D215" s="8"/>
       <c r="E215" s="8"/>
       <c r="F215" s="8">
         <v>10</v>
       </c>
-      <c r="G215" s="26"/>
+      <c r="G215" s="32"/>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A216" s="7"/>
@@ -4109,60 +4106,60 @@
       <c r="F216" s="8">
         <v>10</v>
       </c>
-      <c r="G216" s="26"/>
+      <c r="G216" s="32"/>
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A217" s="7"/>
       <c r="B217" s="7"/>
       <c r="C217" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D217" s="8"/>
       <c r="E217" s="8"/>
       <c r="F217" s="8">
         <v>5</v>
       </c>
-      <c r="G217" s="26"/>
+      <c r="G217" s="32"/>
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A218" s="7"/>
       <c r="B218" s="7"/>
       <c r="C218" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D218" s="8"/>
       <c r="E218" s="8"/>
       <c r="F218" s="8">
         <v>5</v>
       </c>
-      <c r="G218" s="26"/>
+      <c r="G218" s="32"/>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A219" s="7"/>
       <c r="B219" s="7"/>
       <c r="C219" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D219" s="8"/>
       <c r="E219" s="8"/>
       <c r="F219" s="8">
         <v>5</v>
       </c>
-      <c r="G219" s="26"/>
+      <c r="G219" s="32"/>
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A220" s="7"/>
       <c r="B220" s="7"/>
       <c r="C220" s="8"/>
       <c r="D220" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E220" s="15">
         <f>-SUM(E214:E219)</f>
         <v>0</v>
       </c>
       <c r="F220" s="8"/>
-      <c r="G220" s="26"/>
+      <c r="G220" s="32"/>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A221" s="1"/>
@@ -4175,16 +4172,16 @@
         <f>SUM(F214:F219)</f>
         <v>40</v>
       </c>
-      <c r="G221" s="26"/>
+      <c r="G221" s="32"/>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A222" s="1"/>
       <c r="B222" s="1"/>
-      <c r="G222" s="26"/>
+      <c r="G222" s="32"/>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A223" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B223" s="7"/>
       <c r="C223" s="8" t="s">
@@ -4195,22 +4192,22 @@
       <c r="F223" s="8">
         <v>5</v>
       </c>
-      <c r="G223" s="26"/>
+      <c r="G223" s="32"/>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A224" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B224" s="7"/>
       <c r="C224" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D224" s="8"/>
       <c r="E224" s="8"/>
       <c r="F224" s="8">
         <v>25</v>
       </c>
-      <c r="G224" s="26"/>
+      <c r="G224" s="32"/>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A225" s="7"/>
@@ -4223,60 +4220,60 @@
       <c r="F225" s="8">
         <v>15</v>
       </c>
-      <c r="G225" s="26"/>
+      <c r="G225" s="32"/>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A226" s="7"/>
       <c r="B226" s="7"/>
       <c r="C226" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D226" s="8"/>
       <c r="E226" s="8"/>
       <c r="F226" s="8">
         <v>15</v>
       </c>
-      <c r="G226" s="26"/>
+      <c r="G226" s="32"/>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A227" s="7"/>
       <c r="B227" s="7"/>
       <c r="C227" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D227" s="8"/>
       <c r="E227" s="8"/>
       <c r="F227" s="8">
         <v>20</v>
       </c>
-      <c r="G227" s="26"/>
+      <c r="G227" s="32"/>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A228" s="7"/>
       <c r="B228" s="7"/>
       <c r="C228" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D228" s="8"/>
       <c r="E228" s="8"/>
       <c r="F228" s="8">
         <v>15</v>
       </c>
-      <c r="G228" s="26"/>
+      <c r="G228" s="32"/>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A229" s="7"/>
       <c r="B229" s="7"/>
       <c r="C229" s="8"/>
       <c r="D229" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E229" s="15">
         <f>-SUM(E223:E228)</f>
         <v>0</v>
       </c>
       <c r="F229" s="8"/>
-      <c r="G229" s="26"/>
+      <c r="G229" s="32"/>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A230" s="1"/>
@@ -4289,19 +4286,19 @@
         <f>SUM(F223:F228)</f>
         <v>95</v>
       </c>
-      <c r="G230" s="26"/>
+      <c r="G230" s="32"/>
     </row>
     <row r="232" spans="1:7" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A232" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A234" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B234" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C234" s="8"/>
       <c r="D234" s="8"/>
@@ -4315,7 +4312,7 @@
         <v>45</v>
       </c>
       <c r="B235" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C235" s="8"/>
       <c r="D235" s="8"/>
@@ -4327,7 +4324,7 @@
     <row r="236" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A236" s="7"/>
       <c r="B236" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C236" s="8"/>
       <c r="D236" s="8"/>
@@ -4339,7 +4336,7 @@
     <row r="237" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A237" s="7"/>
       <c r="B237" s="8" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C237" s="8"/>
       <c r="D237" s="8"/>
@@ -4351,7 +4348,7 @@
     <row r="238" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A238" s="7"/>
       <c r="B238" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C238" s="8"/>
       <c r="D238" s="8"/>
@@ -4363,10 +4360,10 @@
     <row r="239" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A239" s="7"/>
       <c r="B239" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C239" s="8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D239" s="8"/>
       <c r="E239" s="8"/>
@@ -4378,7 +4375,7 @@
       <c r="A240" s="7"/>
       <c r="B240" s="7"/>
       <c r="C240" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D240" s="8"/>
       <c r="E240" s="8"/>
@@ -4390,7 +4387,7 @@
       <c r="A241" s="7"/>
       <c r="B241" s="7"/>
       <c r="C241" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D241" s="8"/>
       <c r="E241" s="8"/>
@@ -4402,7 +4399,7 @@
       <c r="A242" s="7"/>
       <c r="B242" s="7"/>
       <c r="C242" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D242" s="8"/>
       <c r="E242" s="8"/>
@@ -4414,7 +4411,7 @@
       <c r="A243" s="7"/>
       <c r="B243" s="7"/>
       <c r="C243" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D243" s="8"/>
       <c r="E243" s="8"/>
@@ -4426,7 +4423,7 @@
       <c r="A244" s="7"/>
       <c r="B244" s="7"/>
       <c r="C244" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D244" s="8"/>
       <c r="E244" s="8"/>
@@ -4438,10 +4435,10 @@
       <c r="A245" s="7"/>
       <c r="B245" s="7"/>
       <c r="C245" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D245" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E245" s="8"/>
       <c r="F245" s="8">
@@ -4453,7 +4450,7 @@
       <c r="B246" s="7"/>
       <c r="C246" s="8"/>
       <c r="D246" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E246" s="8"/>
       <c r="F246" s="8">
@@ -4465,7 +4462,7 @@
       <c r="B247" s="7"/>
       <c r="C247" s="8"/>
       <c r="D247" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E247" s="8"/>
       <c r="F247" s="8">
@@ -4477,7 +4474,7 @@
       <c r="B248" s="7"/>
       <c r="C248" s="8"/>
       <c r="D248" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E248" s="8"/>
       <c r="F248" s="8">
@@ -4489,7 +4486,7 @@
       <c r="B249" s="7"/>
       <c r="C249" s="8"/>
       <c r="D249" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E249" s="8"/>
       <c r="F249" s="8">
@@ -4501,7 +4498,7 @@
       <c r="B250" s="7"/>
       <c r="C250" s="8"/>
       <c r="D250" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E250" s="15">
         <f>-SUM(E239:E249)</f>
@@ -4526,10 +4523,10 @@
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A256" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B256" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C256" s="8"/>
       <c r="D256" s="8"/>
@@ -4540,11 +4537,11 @@
     </row>
     <row r="257" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A257" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B257" s="7"/>
       <c r="C257" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D257" s="8"/>
       <c r="E257" s="8"/>
@@ -4556,7 +4553,7 @@
       <c r="A258" s="7"/>
       <c r="B258" s="7"/>
       <c r="C258" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D258" s="8"/>
       <c r="E258" s="8"/>
@@ -4568,7 +4565,7 @@
       <c r="A259" s="7"/>
       <c r="B259" s="7"/>
       <c r="C259" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D259" s="8"/>
       <c r="E259" s="8"/>
@@ -4580,7 +4577,7 @@
       <c r="A260" s="7"/>
       <c r="B260" s="7"/>
       <c r="C260" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D260" s="8"/>
       <c r="E260" s="8"/>
@@ -4591,10 +4588,10 @@
     <row r="261" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A261" s="7"/>
       <c r="B261" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C261" s="8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D261" s="8"/>
       <c r="E261" s="8"/>
@@ -4606,7 +4603,7 @@
       <c r="A262" s="7"/>
       <c r="B262" s="7"/>
       <c r="C262" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D262" s="8"/>
       <c r="E262" s="8"/>
@@ -4618,7 +4615,7 @@
       <c r="A263" s="7"/>
       <c r="B263" s="7"/>
       <c r="C263" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D263" s="8"/>
       <c r="E263" s="8"/>
@@ -4630,7 +4627,7 @@
       <c r="A264" s="7"/>
       <c r="B264" s="7"/>
       <c r="C264" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D264" s="8"/>
       <c r="E264" s="8"/>
@@ -4642,7 +4639,7 @@
       <c r="A265" s="7"/>
       <c r="B265" s="7"/>
       <c r="C265" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D265" s="8"/>
       <c r="E265" s="8"/>
@@ -4654,10 +4651,10 @@
       <c r="A266" s="7"/>
       <c r="B266" s="7"/>
       <c r="C266" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D266" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E266" s="8"/>
       <c r="F266" s="8">
@@ -4669,7 +4666,7 @@
       <c r="B267" s="7"/>
       <c r="C267" s="8"/>
       <c r="D267" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E267" s="8"/>
       <c r="F267" s="8">
@@ -4681,7 +4678,7 @@
       <c r="B268" s="7"/>
       <c r="C268" s="8"/>
       <c r="D268" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E268" s="8"/>
       <c r="F268" s="8">
@@ -4693,7 +4690,7 @@
       <c r="B269" s="7"/>
       <c r="C269" s="8"/>
       <c r="D269" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E269" s="8"/>
       <c r="F269" s="8">
@@ -4705,7 +4702,7 @@
       <c r="B270" s="7"/>
       <c r="C270" s="8"/>
       <c r="D270" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E270" s="8"/>
       <c r="F270" s="8">
@@ -4717,7 +4714,7 @@
       <c r="B271" s="8"/>
       <c r="C271" s="8"/>
       <c r="D271" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E271" s="15">
         <f>-SUM(E256:E260)</f>
@@ -4739,11 +4736,11 @@
     </row>
     <row r="273" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A273" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B273" s="7"/>
       <c r="C273" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D273" s="8"/>
       <c r="E273" s="8" t="s">
@@ -4757,7 +4754,7 @@
       <c r="A274" s="8"/>
       <c r="B274" s="8"/>
       <c r="C274" s="8" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D274" s="8"/>
       <c r="E274" s="8"/>
@@ -4769,7 +4766,7 @@
       <c r="A275" s="7"/>
       <c r="B275" s="8"/>
       <c r="C275" s="8" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D275" s="8"/>
       <c r="E275" s="8"/>
@@ -4781,7 +4778,7 @@
       <c r="A276" s="8"/>
       <c r="B276" s="8"/>
       <c r="C276" s="8" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D276" s="8"/>
       <c r="E276" s="8" t="s">
@@ -4795,7 +4792,7 @@
       <c r="A277" s="8"/>
       <c r="B277" s="8"/>
       <c r="C277" s="8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D277" s="8"/>
       <c r="E277" s="8" t="s">
@@ -4809,7 +4806,7 @@
       <c r="A278" s="7"/>
       <c r="B278" s="8"/>
       <c r="C278" s="8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D278" s="8"/>
       <c r="E278" s="8" t="s">
@@ -4823,7 +4820,7 @@
       <c r="A279" s="7"/>
       <c r="B279" s="8"/>
       <c r="C279" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D279" s="8"/>
       <c r="E279" s="8" t="s">
@@ -4838,7 +4835,7 @@
       <c r="B280" s="8"/>
       <c r="C280" s="8"/>
       <c r="D280" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E280" s="15">
         <f>-SUM(E273:E279)</f>
@@ -4868,17 +4865,17 @@
     </row>
     <row r="285" spans="1:12" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A285" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K285"/>
       <c r="L285"/>
     </row>
     <row r="286" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A286" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B286" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C286" s="8" t="s">
         <v>4</v>
@@ -4895,7 +4892,7 @@
       <c r="A287" s="8"/>
       <c r="B287" s="8"/>
       <c r="C287" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D287" s="8"/>
       <c r="E287" s="8">
@@ -4909,7 +4906,7 @@
       <c r="A288" s="8"/>
       <c r="B288" s="8"/>
       <c r="C288" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D288" s="8"/>
       <c r="E288" s="8">
@@ -4923,7 +4920,7 @@
       <c r="A289" s="8"/>
       <c r="B289" s="8"/>
       <c r="C289" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D289" s="8"/>
       <c r="E289" s="8">
@@ -4937,7 +4934,7 @@
       <c r="A290" s="8"/>
       <c r="B290" s="8"/>
       <c r="C290" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D290" s="8"/>
       <c r="E290" s="8">
@@ -4951,7 +4948,7 @@
       <c r="A291" s="8"/>
       <c r="B291" s="8"/>
       <c r="C291" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D291" s="8"/>
       <c r="E291" s="8">
@@ -4966,7 +4963,7 @@
       <c r="B292" s="8"/>
       <c r="C292" s="8"/>
       <c r="D292" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E292" s="15">
         <f>-SUM(E286:E291)</f>
@@ -4990,7 +4987,7 @@
       </c>
       <c r="B294" s="7"/>
       <c r="C294" s="21" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D294" s="8"/>
       <c r="E294" s="8"/>
@@ -5002,7 +4999,7 @@
       <c r="A295" s="7"/>
       <c r="B295" s="7"/>
       <c r="C295" s="21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D295" s="8"/>
       <c r="E295" s="8"/>
@@ -5014,7 +5011,7 @@
       <c r="A296" s="7"/>
       <c r="B296" s="7"/>
       <c r="C296" s="21" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D296" s="8"/>
       <c r="E296" s="8"/>
@@ -5035,7 +5032,7 @@
       <c r="B298" s="7"/>
       <c r="C298" s="8"/>
       <c r="D298" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E298" s="15">
         <f>-SUM(E294:E297)</f>
@@ -5058,15 +5055,15 @@
     </row>
     <row r="302" spans="1:13" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A302" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="303" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A303" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B303" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C303" s="8"/>
       <c r="D303" s="8"/>
@@ -5078,7 +5075,7 @@
     <row r="304" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A304" s="7"/>
       <c r="B304" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C304" s="8"/>
       <c r="D304" s="8"/>
@@ -5090,7 +5087,7 @@
     <row r="305" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A305" s="7"/>
       <c r="B305" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C305" s="8"/>
       <c r="D305" s="8"/>
@@ -5102,10 +5099,10 @@
     <row r="306" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A306" s="7"/>
       <c r="B306" s="8" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C306" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D306" s="8"/>
       <c r="E306" s="8"/>
@@ -5117,7 +5114,7 @@
       <c r="A307" s="7"/>
       <c r="B307" s="8"/>
       <c r="C307" s="8" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D307" s="8"/>
       <c r="E307" s="8"/>
@@ -5128,10 +5125,10 @@
     <row r="308" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A308" s="7"/>
       <c r="B308" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C308" s="8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D308" s="8"/>
       <c r="E308" s="8"/>
@@ -5143,7 +5140,7 @@
       <c r="A309" s="7"/>
       <c r="B309" s="8"/>
       <c r="C309" s="8" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D309" s="8"/>
       <c r="E309" s="8"/>
@@ -5155,7 +5152,7 @@
       <c r="A310" s="7"/>
       <c r="B310" s="8"/>
       <c r="C310" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D310" s="8"/>
       <c r="E310" s="8"/>
@@ -5167,7 +5164,7 @@
       <c r="A311" s="7"/>
       <c r="B311" s="8"/>
       <c r="C311" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D311" s="8"/>
       <c r="E311" s="8"/>
@@ -5179,7 +5176,7 @@
       <c r="A312" s="7"/>
       <c r="B312" s="8"/>
       <c r="C312" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D312" s="8"/>
       <c r="E312" s="8"/>
@@ -5192,7 +5189,7 @@
       <c r="B313" s="8"/>
       <c r="C313" s="8"/>
       <c r="D313" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E313" s="15">
         <f>-SUM(E255:E312)</f>
@@ -5216,10 +5213,10 @@
     </row>
     <row r="316" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A316" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B316" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C316" s="8"/>
       <c r="D316" s="8"/>
@@ -5227,14 +5224,14 @@
       <c r="F316" s="8">
         <v>100</v>
       </c>
-      <c r="H316" s="27" t="s">
-        <v>51</v>
+      <c r="H316" s="33" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A317" s="8"/>
       <c r="B317" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C317" s="8"/>
       <c r="D317" s="8"/>
@@ -5242,12 +5239,12 @@
       <c r="F317" s="8">
         <v>100</v>
       </c>
-      <c r="H317" s="27"/>
+      <c r="H317" s="33"/>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A318" s="8"/>
       <c r="B318" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C318" s="8"/>
       <c r="D318" s="8"/>
@@ -5255,12 +5252,12 @@
       <c r="F318" s="8">
         <v>100</v>
       </c>
-      <c r="H318" s="27"/>
+      <c r="H318" s="33"/>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A319" s="8"/>
       <c r="B319" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C319" s="8"/>
       <c r="D319" s="8"/>
@@ -5268,23 +5265,23 @@
       <c r="F319" s="8">
         <v>100</v>
       </c>
-      <c r="H319" s="27"/>
+      <c r="H319" s="33"/>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A320" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B320" s="8"/>
       <c r="C320" s="8"/>
       <c r="D320" s="8"/>
       <c r="E320" s="8"/>
       <c r="F320" s="8"/>
-      <c r="H320" s="27"/>
+      <c r="H320" s="33"/>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A321" s="7"/>
       <c r="B321" s="8" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C321" s="8"/>
       <c r="D321" s="8"/>
@@ -5292,12 +5289,12 @@
       <c r="F321" s="8">
         <v>50</v>
       </c>
-      <c r="H321" s="27"/>
+      <c r="H321" s="33"/>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A322" s="8"/>
       <c r="B322" s="8" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C322" s="8"/>
       <c r="D322" s="8"/>
@@ -5307,12 +5304,12 @@
       <c r="F322" s="8">
         <v>0</v>
       </c>
-      <c r="H322" s="27"/>
+      <c r="H322" s="33"/>
     </row>
     <row r="323" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A323" s="8"/>
       <c r="B323" s="8" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C323" s="8"/>
       <c r="D323" s="8"/>
@@ -5322,12 +5319,12 @@
       <c r="F323" s="8">
         <v>0</v>
       </c>
-      <c r="H323" s="27"/>
+      <c r="H323" s="33"/>
     </row>
     <row r="324" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A324" s="8"/>
       <c r="B324" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C324" s="8"/>
       <c r="D324" s="8"/>
@@ -5337,7 +5334,7 @@
       <c r="F324" s="8">
         <v>100</v>
       </c>
-      <c r="H324" s="27"/>
+      <c r="H324" s="33"/>
     </row>
     <row r="325" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A325" s="8"/>
@@ -5346,21 +5343,21 @@
       <c r="D325" s="8"/>
       <c r="E325" s="8"/>
       <c r="F325" s="8"/>
-      <c r="H325" s="27"/>
+      <c r="H325" s="33"/>
     </row>
     <row r="326" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A326" s="8"/>
       <c r="B326" s="8"/>
       <c r="C326" s="8"/>
       <c r="D326" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E326" s="15">
         <f>-SUM(E316:E321)</f>
         <v>0</v>
       </c>
       <c r="F326" s="8"/>
-      <c r="H326" s="27"/>
+      <c r="H326" s="33"/>
     </row>
     <row r="327" spans="1:8" x14ac:dyDescent="0.45">
       <c r="E327">
@@ -5371,19 +5368,19 @@
         <f>SUM(F316:F325)</f>
         <v>550</v>
       </c>
-      <c r="H327" s="27"/>
+      <c r="H327" s="33"/>
     </row>
     <row r="328" spans="1:8" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A328" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="329" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A329" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B329" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C329" s="8"/>
       <c r="D329" s="8"/>
@@ -5397,7 +5394,7 @@
     <row r="330" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A330" s="8"/>
       <c r="B330" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C330" s="8"/>
       <c r="D330" s="8"/>
@@ -5411,7 +5408,7 @@
     <row r="331" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A331" s="8"/>
       <c r="B331" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C331" s="8"/>
       <c r="D331" s="8"/>
@@ -5423,7 +5420,7 @@
     <row r="332" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A332" s="8"/>
       <c r="B332" s="8" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C332" s="8"/>
       <c r="D332" s="8"/>
@@ -5437,7 +5434,7 @@
     <row r="333" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A333" s="8"/>
       <c r="B333" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C333" s="8"/>
       <c r="D333" s="8"/>
@@ -5449,7 +5446,7 @@
     <row r="334" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A334" s="8"/>
       <c r="B334" s="8" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C334" s="8"/>
       <c r="D334" s="8"/>
@@ -5463,7 +5460,7 @@
     <row r="335" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A335" s="8"/>
       <c r="B335" s="8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C335" s="8"/>
       <c r="D335" s="8"/>
@@ -5475,7 +5472,7 @@
     <row r="336" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A336" s="8"/>
       <c r="B336" s="8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C336" s="8"/>
       <c r="D336" s="8"/>
@@ -5489,7 +5486,7 @@
       <c r="B337" s="8"/>
       <c r="C337" s="8"/>
       <c r="D337" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E337" s="15">
         <f>-SUM(E329:E336)*0</f>
@@ -5512,7 +5509,7 @@
         <v>11</v>
       </c>
       <c r="B340" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C340" s="8"/>
       <c r="D340" s="8"/>
@@ -5526,7 +5523,7 @@
     <row r="341" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A341" s="8"/>
       <c r="B341" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C341" s="8"/>
       <c r="D341" s="8"/>
@@ -5540,7 +5537,7 @@
     <row r="342" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A342" s="8"/>
       <c r="B342" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C342" s="8"/>
       <c r="D342" s="8"/>
@@ -5570,7 +5567,7 @@
       <c r="B344" s="8"/>
       <c r="C344" s="8"/>
       <c r="D344" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E344" s="15">
         <f>-SUM(E340:E343)*0</f>
@@ -5592,14 +5589,14 @@
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A346" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B346" s="7"/>
       <c r="C346" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="D346" s="8" t="s">
         <v>222</v>
-      </c>
-      <c r="D346" s="8" t="s">
-        <v>224</v>
       </c>
       <c r="E346" s="8">
         <v>-20</v>
@@ -5613,7 +5610,7 @@
       <c r="B347" s="7"/>
       <c r="C347" s="8"/>
       <c r="D347" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E347" s="8">
         <v>-20</v>
@@ -5627,7 +5624,7 @@
       <c r="B348" s="7"/>
       <c r="C348" s="8"/>
       <c r="D348" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E348" s="8">
         <v>-20</v>
@@ -5640,10 +5637,10 @@
       <c r="A349" s="7"/>
       <c r="B349" s="7"/>
       <c r="C349" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D349" s="8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E349" s="8">
         <v>-20</v>
@@ -5656,10 +5653,10 @@
       <c r="A350" s="7"/>
       <c r="B350" s="7"/>
       <c r="C350" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D350" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E350" s="8">
         <v>-20</v>
@@ -5673,7 +5670,7 @@
       <c r="B351" s="7"/>
       <c r="C351" s="8"/>
       <c r="D351" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E351" s="8">
         <v>-20</v>
@@ -5687,7 +5684,7 @@
       <c r="B352" s="7"/>
       <c r="C352" s="8"/>
       <c r="D352" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E352" s="8">
         <v>-20</v>
@@ -5701,7 +5698,7 @@
       <c r="B353" s="7"/>
       <c r="C353" s="8"/>
       <c r="D353" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E353" s="8">
         <v>0</v>
@@ -5722,18 +5719,18 @@
     </row>
     <row r="355" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A355" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A356" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B356" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C356" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D356" s="8"/>
       <c r="E356" s="8"/>
@@ -5745,7 +5742,7 @@
       <c r="A357" s="7"/>
       <c r="B357" s="8"/>
       <c r="C357" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D357" s="8"/>
       <c r="E357" s="8"/>
@@ -5756,10 +5753,10 @@
     <row r="358" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A358" s="8"/>
       <c r="B358" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C358" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D358" s="8"/>
       <c r="E358" s="8"/>
@@ -5771,7 +5768,7 @@
       <c r="A359" s="8"/>
       <c r="B359" s="8"/>
       <c r="C359" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D359" s="8"/>
       <c r="E359" s="8"/>
@@ -5783,7 +5780,7 @@
       <c r="A360" s="8"/>
       <c r="B360" s="8"/>
       <c r="C360" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D360" s="8"/>
       <c r="E360" s="8"/>
@@ -5795,7 +5792,7 @@
       <c r="A361" s="8"/>
       <c r="B361" s="8"/>
       <c r="C361" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D361" s="8"/>
       <c r="E361" s="8"/>
@@ -5807,7 +5804,7 @@
       <c r="A362" s="8"/>
       <c r="B362" s="8"/>
       <c r="C362" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D362" s="8"/>
       <c r="E362" s="8"/>
@@ -5820,7 +5817,7 @@
       <c r="B363" s="8"/>
       <c r="C363" s="8"/>
       <c r="D363" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E363" s="15">
         <f>-SUM(E360:E362)</f>
@@ -5839,15 +5836,15 @@
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A365" s="1" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A366" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B366" s="8" t="s">
         <v>238</v>
-      </c>
-      <c r="B366" s="8" t="s">
-        <v>240</v>
       </c>
       <c r="C366" s="8"/>
       <c r="D366" s="8"/>
@@ -5860,13 +5857,13 @@
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A367" s="7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B367" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C367" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D367" s="8"/>
       <c r="E367" s="8">
@@ -5880,7 +5877,7 @@
       <c r="A368" s="7"/>
       <c r="B368" s="8"/>
       <c r="C368" s="8" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D368" s="8"/>
       <c r="E368" s="8">
@@ -5895,7 +5892,7 @@
       <c r="B369" s="8"/>
       <c r="C369" s="8"/>
       <c r="D369" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E369" s="15">
         <f>-SUM(E361:E368)</f>
@@ -5923,7 +5920,7 @@
         <v>46</v>
       </c>
       <c r="B373" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C373" s="8"/>
       <c r="D373" s="8"/>
@@ -5935,7 +5932,7 @@
     <row r="374" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A374" s="7"/>
       <c r="B374" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C374" s="8"/>
       <c r="D374" s="8"/>
@@ -5947,7 +5944,7 @@
     <row r="375" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A375" s="7"/>
       <c r="B375" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C375" s="8"/>
       <c r="D375" s="8"/>
@@ -5959,7 +5956,7 @@
     <row r="376" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A376" s="7"/>
       <c r="B376" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C376" s="8"/>
       <c r="D376" s="8"/>
@@ -5971,7 +5968,7 @@
     <row r="377" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A377" s="7"/>
       <c r="B377" s="7" t="s">
-        <v>47</v>
+        <v>298</v>
       </c>
       <c r="C377" s="8"/>
       <c r="D377" s="8"/>
@@ -5983,7 +5980,7 @@
     <row r="378" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A378" s="7"/>
       <c r="B378" s="7" t="s">
-        <v>48</v>
+        <v>297</v>
       </c>
       <c r="C378" s="8"/>
       <c r="D378" s="8"/>
@@ -5995,7 +5992,7 @@
     <row r="379" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A379" s="7"/>
       <c r="B379" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C379" s="8"/>
       <c r="D379" s="8"/>
@@ -6007,7 +6004,7 @@
     <row r="380" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A380" s="7"/>
       <c r="B380" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C380" s="8"/>
       <c r="D380" s="8"/>
@@ -6021,7 +6018,7 @@
       <c r="B381" s="7"/>
       <c r="C381" s="8"/>
       <c r="D381" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E381" s="15">
         <f>-SUM(E373:E380)</f>
@@ -6044,7 +6041,7 @@
     <row r="387" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A387" s="7"/>
       <c r="B387" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E387">
         <f>E382+E370+E364+E354+E345+E338+E327+E314+E299+E293+E281+E272+E251+E230+E221+E211+E199+E186+E174+E161+E148+E136+E130+E119+E111+E103+E95+E84+E73+E63+E46</f>
@@ -6062,7 +6059,7 @@
     <row r="388" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A388" s="9"/>
       <c r="B388" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H388" s="13">
         <f>(E388+E387)/(F388+F387)</f>
@@ -6072,7 +6069,7 @@
     <row r="389" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A389" s="10"/>
       <c r="B389" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H389" s="13">
         <f>(E389+E387)/(F389+F387)</f>
@@ -6082,7 +6079,7 @@
     <row r="390" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A390" s="11"/>
       <c r="B390" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H390" s="13">
         <f>(E390+E387)/(F390+F387)</f>
@@ -6092,7 +6089,7 @@
     <row r="391" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A391" s="20"/>
       <c r="B391" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H391" s="13">
         <f>(E391+E387)/(F391+F387)</f>
@@ -6102,7 +6099,7 @@
     <row r="392" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A392" s="22"/>
       <c r="B392" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H392" s="13">
         <f>(E392+E387)/(F392+F387)</f>
@@ -6111,15 +6108,15 @@
     </row>
     <row r="394" spans="1:8" x14ac:dyDescent="0.45">
       <c r="F394" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="G394" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="395" spans="1:8" x14ac:dyDescent="0.45">
       <c r="D395" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G395" t="s">
         <v>31</v>
@@ -6215,7 +6212,7 @@
     </row>
     <row r="406" spans="5:7" x14ac:dyDescent="0.45">
       <c r="E406" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -6256,19 +6253,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" x14ac:dyDescent="0.75">
-      <c r="A1" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="A1" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D4" s="14">
         <v>-1</v>
@@ -6284,7 +6281,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D6" s="14">
         <v>-0.5</v>
@@ -6292,7 +6289,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D7" s="14">
         <v>-0.5</v>
@@ -6300,7 +6297,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D8" s="14">
         <v>-1</v>
@@ -6308,7 +6305,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D9" s="14">
         <v>-1</v>
@@ -6316,7 +6313,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D10" s="14">
         <v>-0.5</v>
@@ -6324,7 +6321,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D11" s="14">
         <v>-0.5</v>
@@ -6332,7 +6329,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D12" s="14">
         <v>-0.5</v>
@@ -6340,7 +6337,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D13" s="14">
         <v>-0.5</v>
@@ -6348,7 +6345,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D14" s="14">
         <v>-1</v>
@@ -6356,7 +6353,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D15" s="14">
         <v>-0.3</v>
@@ -6364,7 +6361,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D16" s="14">
         <v>-1</v>
@@ -6372,7 +6369,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D17" s="14">
         <v>-0.2</v>
@@ -6380,7 +6377,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D18" s="14">
         <v>-1</v>

</xml_diff>